<commit_message>
classes modals are added.
</commit_message>
<xml_diff>
--- a/DB/Claim_Calling_Tracker.xlsx
+++ b/DB/Claim_Calling_Tracker.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\GitHub\Caller_Tracker\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1722604-2478-4C97-83CF-23EF0C2C1405}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BBBFDEC-0F05-4E91-B8D6-B037711E15C6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Claims" sheetId="1" r:id="rId1"/>
@@ -23,21 +23,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t>ClaimID</t>
   </si>
   <si>
-    <t>CallerLocation</t>
+    <t>ClaimSite</t>
+  </si>
+  <si>
+    <t>ClaimProviderName</t>
+  </si>
+  <si>
+    <t>ClaimQuery</t>
+  </si>
+  <si>
+    <t>ClaimCreationDate</t>
   </si>
   <si>
     <t>ClaimStatus</t>
   </si>
   <si>
-    <t>CallingAttempted</t>
-  </si>
-  <si>
-    <t>UpdatedLocation</t>
+    <t>Attempt</t>
+  </si>
+  <si>
+    <t>ClaimUpdatedSite</t>
   </si>
   <si>
     <t>ClaimInsertionDate</t>
@@ -46,6 +55,18 @@
     <t>ClaimInsertedBy</t>
   </si>
   <si>
+    <t>LastUpdatedDate</t>
+  </si>
+  <si>
+    <t>LastUpdatedBy</t>
+  </si>
+  <si>
+    <t>LastComment</t>
+  </si>
+  <si>
+    <t>ClaimClosedDate</t>
+  </si>
+  <si>
     <t>HistoryID</t>
   </si>
   <si>
@@ -103,7 +124,7 @@
     <t>AppVersion</t>
   </si>
   <si>
-    <t>1.0</t>
+    <t>1.1</t>
   </si>
   <si>
     <t>NextHistoryID</t>
@@ -128,9 +149,6 @@
   </si>
   <si>
     <t>Gurgaon</t>
-  </si>
-  <si>
-    <t>Pending</t>
   </si>
 </sst>
 </file>
@@ -178,12 +196,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -202,16 +219,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:G3">
-  <autoFilter ref="A1:G3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N2">
+  <autoFilter ref="A1:N2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ClaimID"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="CallerLocation"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="ClaimStatus"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="CallingAttempted"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="UpdatedLocation"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ClaimInsertionDate"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="ClaimInsertedBy"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ClaimSite"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="ClaimProviderName"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="ClaimQuery"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="ClaimCreationDate"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="ClaimStatus"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Attempt"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="ClaimUpdatedSite"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="ClaimInsertionDate"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="ClaimInsertedBy"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="LastUpdatedDate"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="LastUpdatedBy"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="LastComment"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ClaimClosedDate"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -517,20 +541,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="32.140625" customWidth="1"/>
-    <col min="7" max="7" width="19" customWidth="1"/>
+    <col min="1" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
+    <col min="6" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="11" width="19" customWidth="1"/>
+    <col min="12" max="12" width="17" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -552,28 +579,26 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>123456</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46274.444155092591</v>
-      </c>
-      <c r="G3" t="s">
-        <v>33</v>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -586,7 +611,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -597,22 +621,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -625,63 +649,62 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -691,48 +714,47 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
app is working fine now
</commit_message>
<xml_diff>
--- a/DB/Claim_Calling_Tracker.xlsx
+++ b/DB/Claim_Calling_Tracker.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\GitHub\Caller_Tracker\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BBBFDEC-0F05-4E91-B8D6-B037711E15C6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{453A8150-4916-4EF7-8E1E-0FA5A4B46E74}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Claims" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,12 @@
     <sheet name="Users" sheetId="3" r:id="rId3"/>
     <sheet name="Config" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" calcMode="manual"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
   <si>
     <t>ClaimID</t>
   </si>
@@ -149,6 +149,45 @@
   </si>
   <si>
     <t>Gurgaon</t>
+  </si>
+  <si>
+    <t>Claim Id1234</t>
+  </si>
+  <si>
+    <t>Noida</t>
+  </si>
+  <si>
+    <t>Provider1</t>
+  </si>
+  <si>
+    <t>Query1</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>ClaimId1111</t>
+  </si>
+  <si>
+    <t>Provider2</t>
+  </si>
+  <si>
+    <t>Query2</t>
+  </si>
+  <si>
+    <t>No Caller attempted the call</t>
+  </si>
+  <si>
+    <t>Claim Id not found</t>
+  </si>
+  <si>
+    <t>Not Reachable</t>
+  </si>
+  <si>
+    <t>Amount recieved</t>
+  </si>
+  <si>
+    <t>Closed</t>
   </si>
 </sst>
 </file>
@@ -196,11 +235,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -219,8 +260,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N2">
-  <autoFilter ref="A1:N2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N4">
+  <autoFilter ref="A1:N4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ClaimID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ClaimSite"/>
@@ -242,8 +283,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F2">
-  <autoFilter ref="A1:F2" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F6">
+  <autoFilter ref="A1:F6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="HistoryID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="ClaimID"/>
@@ -541,7 +582,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N1"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -601,6 +643,82 @@
         <v>13</v>
       </c>
     </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="2">
+        <v>46023</v>
+      </c>
+      <c r="F3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="3">
+        <v>46274.647858796299</v>
+      </c>
+      <c r="J3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="2">
+        <v>46055</v>
+      </c>
+      <c r="F4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="3">
+        <v>46274.649594907409</v>
+      </c>
+      <c r="J4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" s="3">
+        <v>46274.655821759261</v>
+      </c>
+      <c r="L4" t="s">
+        <v>40</v>
+      </c>
+      <c r="M4" t="s">
+        <v>53</v>
+      </c>
+      <c r="N4" s="3">
+        <v>46274.655821759261</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -611,7 +729,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F1"/>
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="16" customWidth="1"/>
@@ -639,6 +758,86 @@
         <v>18</v>
       </c>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="3">
+        <v>46274.654467592591</v>
+      </c>
+      <c r="E3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="3">
+        <v>46274.65552083333</v>
+      </c>
+      <c r="E4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="3">
+        <v>46274.655671296299</v>
+      </c>
+      <c r="E5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="3">
+        <v>46274.655821759261</v>
+      </c>
+      <c r="E6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" t="s">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -649,6 +848,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -714,6 +914,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Adding modules is fine.
</commit_message>
<xml_diff>
--- a/DB/Claim_Calling_Tracker.xlsx
+++ b/DB/Claim_Calling_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\GitHub\Caller_Tracker\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{453A8150-4916-4EF7-8E1E-0FA5A4B46E74}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA041A6-F6CE-4111-B0BF-5C2D6B0B0302}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="66">
   <si>
     <t>ClaimID</t>
   </si>
@@ -188,6 +188,39 @@
   </si>
   <si>
     <t>Closed</t>
+  </si>
+  <si>
+    <t>ClaimId12</t>
+  </si>
+  <si>
+    <t>Proiver3</t>
+  </si>
+  <si>
+    <t>Query4</t>
+  </si>
+  <si>
+    <t>ClaimId13</t>
+  </si>
+  <si>
+    <t>Query5</t>
+  </si>
+  <si>
+    <t>ClaimId14</t>
+  </si>
+  <si>
+    <t>Query6</t>
+  </si>
+  <si>
+    <t>ClaimId16</t>
+  </si>
+  <si>
+    <t>Provider5</t>
+  </si>
+  <si>
+    <t>ClaimId18</t>
+  </si>
+  <si>
+    <t>ClaimId19</t>
   </si>
 </sst>
 </file>
@@ -207,6 +240,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -260,8 +294,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N4">
-  <autoFilter ref="A1:N4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N10">
+  <autoFilter ref="A1:N10" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ClaimID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ClaimSite"/>
@@ -583,7 +617,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -717,6 +751,198 @@
       </c>
       <c r="N4" s="3">
         <v>46274.655821759261</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="2">
+        <v>46056</v>
+      </c>
+      <c r="F5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" s="3">
+        <v>46274.685497685183</v>
+      </c>
+      <c r="J5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="2">
+        <v>46056</v>
+      </c>
+      <c r="F6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="3">
+        <v>46274.685497685183</v>
+      </c>
+      <c r="J6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="2">
+        <v>46056</v>
+      </c>
+      <c r="F7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="3">
+        <v>46274.685497685183</v>
+      </c>
+      <c r="J7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="2">
+        <v>46084</v>
+      </c>
+      <c r="F8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" s="3">
+        <v>46274.687141203707</v>
+      </c>
+      <c r="J8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="2">
+        <v>46084</v>
+      </c>
+      <c r="F9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>43</v>
+      </c>
+      <c r="I9" s="3">
+        <v>46274.687141203707</v>
+      </c>
+      <c r="J9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="2">
+        <v>46084</v>
+      </c>
+      <c r="F10" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
+        <v>43</v>
+      </c>
+      <c r="I10" s="3">
+        <v>46274.694351851853</v>
+      </c>
+      <c r="J10" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
module is styled and working well.
</commit_message>
<xml_diff>
--- a/DB/Claim_Calling_Tracker.xlsx
+++ b/DB/Claim_Calling_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\GitHub\Caller_Tracker\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA041A6-F6CE-4111-B0BF-5C2D6B0B0302}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBA0ADC2-05CA-4348-B98D-CD094D7956DC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="69">
   <si>
     <t>ClaimID</t>
   </si>
@@ -221,6 +221,24 @@
   </si>
   <si>
     <t>ClaimId19</t>
+  </si>
+  <si>
+    <t>Claim Query 1</t>
+  </si>
+  <si>
+    <t>Provider4</t>
+  </si>
+  <si>
+    <t>Query 5skfjkdsfjds_x000D_
+sfdsfds_x000D_
+fsdfd_x000D_
+sfd_x000D_
+sf_x000D_
+dsfds_x000D_
+fsdf_x000D_
+sdf_x000D_
+sdf_x000D_
+sd</t>
   </si>
 </sst>
 </file>
@@ -269,13 +287,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -294,8 +315,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N10">
-  <autoFilter ref="A1:N10" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N13">
+  <autoFilter ref="A1:N13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ClaimID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ClaimSite"/>
@@ -617,7 +638,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -942,6 +963,102 @@
         <v>46274.694351851853</v>
       </c>
       <c r="J10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>11223344</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="2">
+        <v>46055</v>
+      </c>
+      <c r="F11" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11" s="3">
+        <v>46275.459710648145</v>
+      </c>
+      <c r="J11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>123123</v>
+      </c>
+      <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" s="2">
+        <v>46055</v>
+      </c>
+      <c r="F12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12" t="s">
+        <v>43</v>
+      </c>
+      <c r="I12" s="3">
+        <v>46275.57476851852</v>
+      </c>
+      <c r="J12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>55555</v>
+      </c>
+      <c r="B13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E13" s="2">
+        <v>46024</v>
+      </c>
+      <c r="F13" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I13" s="3">
+        <v>46275.575266203705</v>
+      </c>
+      <c r="J13" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>

<commit_message>
current app working fine
</commit_message>
<xml_diff>
--- a/DB/Claim_Calling_Tracker.xlsx
+++ b/DB/Claim_Calling_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\GitHub\Caller_Tracker\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DADFDC-F8AE-4271-BB56-05283A044DD5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6068FF19-32C2-4C30-A13B-0F34D9525999}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="80">
   <si>
     <t>ClaimID</t>
   </si>
@@ -221,9 +221,6 @@
   </si>
   <si>
     <t>ClaimId19</t>
-  </si>
-  <si>
-    <t>Claim Query 1</t>
   </si>
   <si>
     <t>Provider4</t>
@@ -239,6 +236,42 @@
 sdf_x000D_
 sdf_x000D_
 sd</t>
+  </si>
+  <si>
+    <t>Srinivas</t>
+  </si>
+  <si>
+    <t>Query 2 is good one.</t>
+  </si>
+  <si>
+    <t>Sachin</t>
+  </si>
+  <si>
+    <t>Query 3</t>
+  </si>
+  <si>
+    <t>Provider Name5</t>
+  </si>
+  <si>
+    <t>Query 5</t>
+  </si>
+  <si>
+    <t>Chitresh</t>
+  </si>
+  <si>
+    <t>User not at home</t>
+  </si>
+  <si>
+    <t>not found</t>
+  </si>
+  <si>
+    <t>amount recieved</t>
+  </si>
+  <si>
+    <t>Chitresh Pratap Singh</t>
+  </si>
+  <si>
+    <t>Claim Query 10</t>
   </si>
 </sst>
 </file>
@@ -315,8 +348,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N13">
-  <autoFilter ref="A1:N13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N17">
+  <autoFilter ref="A1:N17" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ClaimID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ClaimSite"/>
@@ -338,8 +371,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F6">
-  <autoFilter ref="A1:F6" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F9">
+  <autoFilter ref="A1:F9" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="HistoryID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="ClaimID"/>
@@ -638,7 +671,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -971,13 +1004,13 @@
         <v>11223344</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="E11" s="2">
         <v>46055</v>
@@ -986,16 +1019,25 @@
         <v>46</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="I11" s="3">
         <v>46275.459710648145</v>
       </c>
       <c r="J11" t="s">
         <v>40</v>
+      </c>
+      <c r="K11" s="3">
+        <v>46277.215578703705</v>
+      </c>
+      <c r="L11" t="s">
+        <v>40</v>
+      </c>
+      <c r="M11" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -1006,7 +1048,7 @@
         <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D12" t="s">
         <v>59</v>
@@ -1015,10 +1057,10 @@
         <v>46055</v>
       </c>
       <c r="F12" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H12" t="s">
         <v>41</v>
@@ -1030,10 +1072,16 @@
         <v>40</v>
       </c>
       <c r="K12" s="3">
-        <v>46275.683599537035</v>
+        <v>46277.186168981483</v>
       </c>
       <c r="L12" t="s">
         <v>40</v>
+      </c>
+      <c r="M12" t="s">
+        <v>77</v>
+      </c>
+      <c r="N12" s="3">
+        <v>46277.186168981483</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="165" x14ac:dyDescent="0.25">
@@ -1047,7 +1095,7 @@
         <v>63</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E13" s="2">
         <v>46024</v>
@@ -1065,6 +1113,134 @@
         <v>46275.575266203705</v>
       </c>
       <c r="J13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>1231234</v>
+      </c>
+      <c r="B14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" t="s">
+        <v>69</v>
+      </c>
+      <c r="E14" s="2">
+        <v>46276</v>
+      </c>
+      <c r="F14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="3">
+        <v>46276.529479166667</v>
+      </c>
+      <c r="J14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>4141</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" s="2">
+        <v>414949</v>
+      </c>
+      <c r="F15" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15" t="s">
+        <v>43</v>
+      </c>
+      <c r="I15" s="3">
+        <v>46276.548310185186</v>
+      </c>
+      <c r="J15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>6767</v>
+      </c>
+      <c r="B16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="2">
+        <v>46023</v>
+      </c>
+      <c r="F16" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16" t="s">
+        <v>41</v>
+      </c>
+      <c r="I16" s="3">
+        <v>46276.552395833336</v>
+      </c>
+      <c r="J16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>671234</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" s="2">
+        <v>46023</v>
+      </c>
+      <c r="F17" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>27</v>
+      </c>
+      <c r="I17" s="3">
+        <v>46276.558287037034</v>
+      </c>
+      <c r="J17" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1079,7 +1255,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="16" customWidth="1"/>
@@ -1184,6 +1360,66 @@
         <v>53</v>
       </c>
       <c r="F6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>11223344</v>
+      </c>
+      <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="3">
+        <v>46277.185011574074</v>
+      </c>
+      <c r="E7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>123123</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="3">
+        <v>46277.185833333337</v>
+      </c>
+      <c r="E8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>123123</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="3">
+        <v>46277.186168981483</v>
+      </c>
+      <c r="E9" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" t="s">
         <v>54</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reopening of claim is working fine
</commit_message>
<xml_diff>
--- a/DB/Claim_Calling_Tracker.xlsx
+++ b/DB/Claim_Calling_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\GitHub\Caller_Tracker\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6068FF19-32C2-4C30-A13B-0F34D9525999}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B28F56-ABDC-4783-8806-839416D90D8D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="81">
   <si>
     <t>ClaimID</t>
   </si>
@@ -272,6 +272,9 @@
   </si>
   <si>
     <t>Claim Query 10</t>
+  </si>
+  <si>
+    <t>[REOPENED BY ADMIN] Testing Reason</t>
   </si>
 </sst>
 </file>
@@ -371,8 +374,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F9">
-  <autoFilter ref="A1:F9" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F10">
+  <autoFilter ref="A1:F10" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="HistoryID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="ClaimID"/>
@@ -1057,7 +1060,7 @@
         <v>46055</v>
       </c>
       <c r="F12" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G12">
         <v>2</v>
@@ -1072,17 +1075,15 @@
         <v>40</v>
       </c>
       <c r="K12" s="3">
-        <v>46277.186168981483</v>
+        <v>46277.23883101852</v>
       </c>
       <c r="L12" t="s">
         <v>40</v>
       </c>
       <c r="M12" t="s">
-        <v>77</v>
-      </c>
-      <c r="N12" s="3">
-        <v>46277.186168981483</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="N12" s="3"/>
     </row>
     <row r="13" spans="1:14" ht="165" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -1255,7 +1256,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="16" customWidth="1"/>
@@ -1421,6 +1422,26 @@
       </c>
       <c r="F9" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>123123</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="3">
+        <v>46277.23883101852</v>
+      </c>
+      <c r="E10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>